<commit_message>
fix: Yeşilova ödeme planı Excel'lerinde faiz toplamı hücresi boş
Ledger'da bağımsız bir "toplam faiz" alanı yok — karşılaştırılacak bir
referans değer olmadığı için hiçbir toplam (SUM formülü dahil)
gösterilmemeli. D30'daki =SUM(D15) formülü ve Interest_Total defined
name kaldırıldı; hücre artık boş.

Önce/sonra fark (iki workbook'ta da, yalnız bu hücre): D30 18.240 ->
boş; formül =SUM(D15) -> yok; named ranges 4 -> 3 (Interest_Total
düştü). Taksit #11'in kendi değeri (18.240, D15), diğer taksitlerin
boş hücreleri, "Not" açıklaması ve anapara/durum sütunları değişmedi.

make lint + validate-ledger/documents/excel + make test: yeşil
(622 backend + 18 ocr-worker).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed_data/excel/Yesilova_Repayment_Schedule_2026-03.xlsx
+++ b/seed_data/excel/Yesilova_Repayment_Schedule_2026-03.xlsx
@@ -12,7 +12,6 @@
     <sheet name="_meta" sheetId="2" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="Interest_Total" vbProcedure="false">Schedule!$D$30</definedName>
     <definedName function="false" hidden="false" name="Ledger_DemoToday" vbProcedure="false">_meta!$B$4</definedName>
     <definedName function="false" hidden="false" name="Schedule_LastRow" vbProcedure="false">Schedule!$A$28</definedName>
     <definedName function="false" hidden="false" name="Snapshot_Date" vbProcedure="false">Schedule!$B$2</definedName>
@@ -71,7 +70,7 @@
     <t xml:space="preserve">generated_at</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-10T20:12:49+00:00</t>
+    <t xml:space="preserve">2026-10-11T07:14:19+00:00</t>
   </si>
   <si>
     <t xml:space="preserve">ledger_schema_version</t>
@@ -579,10 +578,6 @@
       <c r="C30" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="D30" s="0" t="n">
-        <f aca="false">SUM(D15)</f>
-        <v>18240</v>
-      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C31" s="0" t="s">

</xml_diff>